<commit_message>
refactor(backend): restructure execution stage and add deterministic short-answer output
</commit_message>
<xml_diff>
--- a/artifacts/output/test4_output.xlsx
+++ b/artifacts/output/test4_output.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -608,22 +608,10 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
           <t>Total Duration (hours)</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B9" t="n">
         <v>14</v>
       </c>
     </row>

</xml_diff>